<commit_message>
Dapine v3.0 FINAL - Standalone EXE with ALL features
</commit_message>
<xml_diff>
--- a/ml_output.xlsx
+++ b/ml_output.xlsx
@@ -59,9 +59,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -495,7 +493,7 @@
         <v>450000</v>
       </c>
       <c r="E3" t="n">
-        <v>400000</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="4">

</xml_diff>